<commit_message>
EWU Portal System- Update Database,Course Management, Advising and Pre-advising
</commit_message>
<xml_diff>
--- a/Common_Course_Schedule_(CSE-ICE-EEE).xlsx
+++ b/Common_Course_Schedule_(CSE-ICE-EEE).xlsx
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="K7" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="K8" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="K9" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="K14" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="K15" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="K16" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="K17" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="K18" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="K19" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="K20" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="K21" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -1755,7 +1755,7 @@
         <v>26</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1802,7 +1802,7 @@
         <v>25</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1849,7 +1849,7 @@
         <v>28</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1896,7 +1896,7 @@
         <v>27</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1943,7 +1943,7 @@
         <v>30</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1990,7 +1990,7 @@
         <v>29</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -2037,7 +2037,7 @@
         <v>32</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2084,7 +2084,7 @@
         <v>31</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="K34" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35">
@@ -2182,7 +2182,7 @@
         </is>
       </c>
       <c r="K35" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36">
@@ -2231,7 +2231,7 @@
         </is>
       </c>
       <c r="K36" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37">
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="K37" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38">
@@ -2327,7 +2327,7 @@
         <v>38</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2374,7 +2374,7 @@
         <v>37</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2421,7 +2421,7 @@
         <v>40</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -2468,7 +2468,7 @@
         <v>39</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2515,7 +2515,7 @@
         <v>42</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2562,7 +2562,7 @@
         <v>41</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -2609,7 +2609,7 @@
         <v>44</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2656,7 +2656,7 @@
         <v>43</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">

</xml_diff>